<commit_message>
Clean public publication files and fix RFdiffusion3 plot legends
Keep preparation inputs and development audits outside the public tree; retain concise analysis notes, final models, measurements, and runnable notebooks. Remove local filesystem locations from saved outputs, workbook metadata, and archived design configurations while preserving scientific data.

Separate substrate and fit-window legends in all 19 standalone RFdiffusion3 kinetics figures. Validate notebook execution, unchanged numerical results, all 234 PTE checks, nine reference figure comparisons, archive metadata, and 88 preserved design metadata files.
</commit_message>
<xml_diff>
--- a/Manuscript_Data/Metallohydrolase_Nature_2026/raw_wetlab_data/240826_zn_hydrolase_donghyo_knockouts_AND_variants_200uM_zn_25uM_PA_AND_100uM_PA.xlsx
+++ b/Manuscript_Data/Metallohydrolase_Nature_2026/raw_wetlab_data/240826_zn_hydrolase_donghyo_knockouts_AND_variants_200uM_zn_25uM_PA_AND_100uM_PA.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Users\Baker_Lab\woodbuse\neo2_platereader\zinc_hydrolase\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{51AD8B0D-D6AA-447E-AF3D-AFE2DB419A5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
@@ -44,13 +39,13 @@
     <t>Experiment File Path:</t>
   </si>
   <si>
-    <t>Z:\Users\Baker_Lab\woodbuse\neo2_platereader\zinc_hydrolase\paper_data\240826_zn_hydrolase_donghyo_knockouts_AND_variants_200uM_zn_25uM_PA_AND_100uM_PA.xpt</t>
+    <t>240826_zn_hydrolase_donghyo_knockouts_AND_variants_200uM_zn_25uM_PA_AND_100uM_PA.xpt</t>
   </si>
   <si>
     <t>Protocol File Path:</t>
   </si>
   <si>
-    <t>Z:\Users\Baker_Lab\woodbuse\neo2_platereader\zinc_hydrolase\4MU_subst_kinetic_SETH.prt</t>
+    <t>4MU_subst_kinetic_SETH.prt</t>
   </si>
   <si>
     <t>Plate Number</t>

</xml_diff>